<commit_message>
Fix md2jcr conversion errors and import term insurance pages at site root
- Table Rounded / Table Comparison: replace per-column-count row models
  (only supported by md2jcr for the built-in Table block) with a single
  4-column row model; block JS drops unused trailing columns
- Cards Video / Cards Quicklinks: rename component titles so md2jcr can
  resolve them ("Cards (Video)" was read as cards + video variant)
- Import scripts write /term-insurance and /term-insurance-redesign at the
  site root so the pages appear in Content Sync

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-life-insurance-plans.report.xlsx
+++ b/tools/importer/reports/import-life-insurance-plans.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="43">
   <si>
     <t>_reportFile</t>
   </si>
@@ -97,25 +97,49 @@
     <t>https://www.nprpl.com/project-gallery-photos</t>
   </si>
   <si>
+    <t>term-insurance.report.json</t>
+  </si>
+  <si>
+    <t>["hero-calculator","cards-pricing","tabs-illustration","cards-plan","cards-plan","cards-icon-list","cards-icon-list","carousel-persona","carousel-persona","embed-video","cards-plan-links","cards-feature-grid","cards-feature-grid","cards-feature-grid","columns-calculator","cards-stats","accordion-seo","accordion-seo","accordion-seo","cards-factor","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-comparison","cards-label-box","cards-label-box","columns-duration","cards-text-tile","cards-text-tile","columns-image-table","carousel-reviews","form-callback","cards-article","tabs-faq"]</t>
+  </si>
+  <si>
+    <t>term-insurance</t>
+  </si>
+  <si>
+    <t>life-insurance-plans</t>
+  </si>
+  <si>
+    <t>2026-10-06T10:08:26.948Z</t>
+  </si>
+  <si>
+    <t>Buy Best Term Insurance Plan &amp; Policy Online in India 2026</t>
+  </si>
+  <si>
+    <t>https://www.tataaia.com/life-insurance-plans/term-insurance.html</t>
+  </si>
+  <si>
+    <t>life-insurance-plans/term-insurance-redesign.report.json</t>
+  </si>
+  <si>
+    <t>["hero-calculator","cards-pricing","cards-plan","cards-plan","cards-icon-list","cards-icon-list","carousel-persona","embed-video","cards-plan-links","cards-feature-grid","cards-feature-grid","cards-feature-grid","columns-calculator","cards-stats","accordion-seo","accordion-seo","accordion-seo","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-comparison","cards-label-box","cards-label-box","columns-duration","cards-text-tile","cards-text-tile","columns-image-table","carousel-reviews","form-callback","cards-article","tabs-faq"]</t>
+  </si>
+  <si>
+    <t>life-insurance-plans/term-insurance-redesign</t>
+  </si>
+  <si>
+    <t>term-insurance-redesign</t>
+  </si>
+  <si>
+    <t>2026-10-06T08:07:37.342Z</t>
+  </si>
+  <si>
     <t>life-insurance-plans/term-insurance.report.json</t>
   </si>
   <si>
-    <t>["hero-calculator","cards-pricing","tabs-illustration","cards-plan","cards-plan","cards-icon-list","cards-icon-list","carousel-persona","carousel-persona","embed-video","cards-plan-links","cards-feature-grid","cards-feature-grid","cards-feature-grid","columns-calculator","cards-stats","accordion-seo","accordion-seo","accordion-seo","cards-factor","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-rounded","table-comparison","cards-label-box","cards-label-box","columns-duration","cards-text-tile","cards-text-tile","columns-image-table","carousel-reviews","form-callback","cards-article","tabs-faq"]</t>
-  </si>
-  <si>
     <t>life-insurance-plans/term-insurance</t>
   </si>
   <si>
-    <t>life-insurance-plans</t>
-  </si>
-  <si>
     <t>2026-10-01T16:37:23.497Z</t>
-  </si>
-  <si>
-    <t>Buy Best Term Insurance Plan &amp; Policy Online in India 2026</t>
-  </si>
-  <si>
-    <t>https://www.tataaia.com/life-insurance-plans/term-insurance.html</t>
   </si>
 </sst>
 </file>
@@ -504,13 +528,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="49" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="37" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="46" customWidth="1"/>
+    <col min="5" max="5" width="25" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
@@ -645,6 +668,58 @@
         <v>34</v>
       </c>
     </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>38</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
+        <v>33</v>
+      </c>
+      <c r="H6" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" t="s">
+        <v>41</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H7" t="s">
+        <v>34</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>